<commit_message>
FY admin website deployment config
</commit_message>
<xml_diff>
--- a/FutureYou/bullhorn/talentMapping/FYTalentMap_Jaybro_Logistics&PurchasingManager_Nov25[38].xlsx
+++ b/FutureYou/bullhorn/talentMapping/FYTalentMap_Jaybro_Logistics&PurchasingManager_Nov25[38].xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://futureyou.sharepoint.com/sites/Group/Shared Documents/Lisa/Jaybro/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leo/Github/XeroAPI/FutureYou/bullhorn/talentMapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{76AB0A8C-60FF-44C1-B6BB-6D63293303CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5136C8C1-54E1-4141-BF5D-147919775B90}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A295C78-70AC-F446-8F96-A0262E35FF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8F154A57-423F-4A68-9F07-D4BFBA117564}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="21440" xr2:uid="{8F154A57-423F-4A68-9F07-D4BFBA117564}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Toll Group</t>
+  </si>
+  <si>
+    <t>This candidate is cool</t>
+  </si>
+  <si>
+    <t>This candidate sux</t>
   </si>
 </sst>
 </file>
@@ -152,7 +158,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -162,6 +168,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -194,12 +212,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -536,16 +555,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77454CDC-1D9F-4B34-9703-54DD06687428}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -568,7 +587,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -587,8 +606,8 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -604,9 +623,11 @@
       <c r="F3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -625,8 +646,8 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -642,19 +663,21 @@
       <c r="F5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="2"/>
@@ -663,17 +686,17 @@
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E7" s="2"/>
@@ -696,6 +719,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f394977a-6c5f-4b10-a16b-c297defcd503">
@@ -704,15 +736,6 @@
     <TaxCatchAll xmlns="37d23ee1-3593-4e12-a3a5-2f3884e9a66a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -971,20 +994,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11C1199E-2582-45AC-ABE0-48BCEEC727E6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A7F202F-5B05-4B79-AA1E-038BDFCAC4C4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="f394977a-6c5f-4b10-a16b-c297defcd503"/>
     <ds:schemaRef ds:uri="37d23ee1-3593-4e12-a3a5-2f3884e9a66a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11C1199E-2582-45AC-ABE0-48BCEEC727E6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>